<commit_message>
Auto update BMKG data
</commit_message>
<xml_diff>
--- a/data/data_suhu_lama.xlsx
+++ b/data/data_suhu_lama.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2470"/>
+  <dimension ref="A1:L2480"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -103066,6 +103066,406 @@
         </is>
       </c>
     </row>
+    <row r="2471">
+      <c r="A2471" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B2471" t="inlineStr">
+        <is>
+          <t>KEDIRI</t>
+        </is>
+      </c>
+      <c r="C2471" t="n">
+        <v>23</v>
+      </c>
+      <c r="D2471" t="n">
+        <v>33</v>
+      </c>
+      <c r="E2471" t="n">
+        <v>26.95</v>
+      </c>
+      <c r="F2471" t="n">
+        <v>63.43</v>
+      </c>
+      <c r="G2471" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2471" t="inlineStr"/>
+      <c r="I2471" t="n">
+        <v>37</v>
+      </c>
+      <c r="J2471" t="n">
+        <v>112</v>
+      </c>
+      <c r="K2471" t="n">
+        <v>21.91</v>
+      </c>
+      <c r="L2471" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="2472">
+      <c r="A2472" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B2472" t="inlineStr">
+        <is>
+          <t>MALANG</t>
+        </is>
+      </c>
+      <c r="C2472" t="n">
+        <v>20</v>
+      </c>
+      <c r="D2472" t="n">
+        <v>32</v>
+      </c>
+      <c r="E2472" t="n">
+        <v>24.43</v>
+      </c>
+      <c r="F2472" t="n">
+        <v>76.05</v>
+      </c>
+      <c r="G2472" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H2472" t="inlineStr"/>
+      <c r="I2472" t="n">
+        <v>37</v>
+      </c>
+      <c r="J2472" t="n">
+        <v>135</v>
+      </c>
+      <c r="K2472" t="n">
+        <v>17.18</v>
+      </c>
+      <c r="L2472" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="2473">
+      <c r="A2473" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B2473" t="inlineStr">
+        <is>
+          <t>PASURUAN</t>
+        </is>
+      </c>
+      <c r="C2473" t="n">
+        <v>19</v>
+      </c>
+      <c r="D2473" t="n">
+        <v>31</v>
+      </c>
+      <c r="E2473" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="F2473" t="n">
+        <v>67.48</v>
+      </c>
+      <c r="G2473" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H2473" t="inlineStr"/>
+      <c r="I2473" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J2473" t="n">
+        <v>112</v>
+      </c>
+      <c r="K2473" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="L2473" t="inlineStr">
+        <is>
+          <t>SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="2474">
+      <c r="A2474" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B2474" t="inlineStr">
+        <is>
+          <t>SIDOARJO</t>
+        </is>
+      </c>
+      <c r="C2474" t="n">
+        <v>24</v>
+      </c>
+      <c r="D2474" t="n">
+        <v>34</v>
+      </c>
+      <c r="E2474" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="F2474" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="G2474" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2474" t="inlineStr"/>
+      <c r="I2474" t="n">
+        <v>37</v>
+      </c>
+      <c r="J2474" t="n">
+        <v>112</v>
+      </c>
+      <c r="K2474" t="n">
+        <v>14.59</v>
+      </c>
+      <c r="L2474" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="2475">
+      <c r="A2475" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B2475" t="inlineStr">
+        <is>
+          <t>SURABAYA</t>
+        </is>
+      </c>
+      <c r="C2475" t="n">
+        <v>24</v>
+      </c>
+      <c r="D2475" t="n">
+        <v>35</v>
+      </c>
+      <c r="E2475" t="n">
+        <v>29.25</v>
+      </c>
+      <c r="F2475" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="G2475" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2475" t="inlineStr"/>
+      <c r="I2475" t="n">
+        <v>37</v>
+      </c>
+      <c r="J2475" t="n">
+        <v>101</v>
+      </c>
+      <c r="K2475" t="n">
+        <v>14.12</v>
+      </c>
+      <c r="L2475" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="2476">
+      <c r="A2476" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B2476" t="inlineStr">
+        <is>
+          <t>KEDIRI</t>
+        </is>
+      </c>
+      <c r="C2476" t="n">
+        <v>23</v>
+      </c>
+      <c r="D2476" t="n">
+        <v>33</v>
+      </c>
+      <c r="E2476" t="n">
+        <v>26.95</v>
+      </c>
+      <c r="F2476" t="n">
+        <v>63.43</v>
+      </c>
+      <c r="G2476" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2476" t="inlineStr"/>
+      <c r="I2476" t="n">
+        <v>37</v>
+      </c>
+      <c r="J2476" t="n">
+        <v>112</v>
+      </c>
+      <c r="K2476" t="n">
+        <v>21.91</v>
+      </c>
+      <c r="L2476" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="2477">
+      <c r="A2477" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B2477" t="inlineStr">
+        <is>
+          <t>MALANG</t>
+        </is>
+      </c>
+      <c r="C2477" t="n">
+        <v>20</v>
+      </c>
+      <c r="D2477" t="n">
+        <v>32</v>
+      </c>
+      <c r="E2477" t="n">
+        <v>24.43</v>
+      </c>
+      <c r="F2477" t="n">
+        <v>76.05</v>
+      </c>
+      <c r="G2477" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H2477" t="inlineStr"/>
+      <c r="I2477" t="n">
+        <v>37</v>
+      </c>
+      <c r="J2477" t="n">
+        <v>135</v>
+      </c>
+      <c r="K2477" t="n">
+        <v>17.18</v>
+      </c>
+      <c r="L2477" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="2478">
+      <c r="A2478" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B2478" t="inlineStr">
+        <is>
+          <t>PASURUAN</t>
+        </is>
+      </c>
+      <c r="C2478" t="n">
+        <v>19</v>
+      </c>
+      <c r="D2478" t="n">
+        <v>31</v>
+      </c>
+      <c r="E2478" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="F2478" t="n">
+        <v>67.48</v>
+      </c>
+      <c r="G2478" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H2478" t="inlineStr"/>
+      <c r="I2478" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J2478" t="n">
+        <v>112</v>
+      </c>
+      <c r="K2478" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="L2478" t="inlineStr">
+        <is>
+          <t>SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="2479">
+      <c r="A2479" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B2479" t="inlineStr">
+        <is>
+          <t>SIDOARJO</t>
+        </is>
+      </c>
+      <c r="C2479" t="n">
+        <v>24</v>
+      </c>
+      <c r="D2479" t="n">
+        <v>34</v>
+      </c>
+      <c r="E2479" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="F2479" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="G2479" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2479" t="inlineStr"/>
+      <c r="I2479" t="n">
+        <v>37</v>
+      </c>
+      <c r="J2479" t="n">
+        <v>112</v>
+      </c>
+      <c r="K2479" t="n">
+        <v>14.59</v>
+      </c>
+      <c r="L2479" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="2480">
+      <c r="A2480" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B2480" t="inlineStr">
+        <is>
+          <t>SURABAYA</t>
+        </is>
+      </c>
+      <c r="C2480" t="n">
+        <v>24</v>
+      </c>
+      <c r="D2480" t="n">
+        <v>35</v>
+      </c>
+      <c r="E2480" t="n">
+        <v>29.25</v>
+      </c>
+      <c r="F2480" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="G2480" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2480" t="inlineStr"/>
+      <c r="I2480" t="n">
+        <v>37</v>
+      </c>
+      <c r="J2480" t="n">
+        <v>101</v>
+      </c>
+      <c r="K2480" t="n">
+        <v>14.12</v>
+      </c>
+      <c r="L2480" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>